<commit_message>
semi-final commit (it can never be finalized)
</commit_message>
<xml_diff>
--- a/fx_pipeline/data/gold/marts/excel/gold_conversion_reference.xlsx
+++ b/fx_pipeline/data/gold/marts/excel/gold_conversion_reference.xlsx
@@ -413,336 +413,183 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>base_currency</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>target_currency</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>base_amount</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>converted_amount</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>1000</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>INR</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>92.81999999999999</v>
+        <v>0.73965</v>
+      </c>
+      <c r="D2" t="n">
+        <v>7.3965</v>
+      </c>
+      <c r="E2" t="n">
+        <v>73.965</v>
+      </c>
+      <c r="F2" t="n">
+        <v>739.65</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>INR</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>10</v>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>928.1999999999999</v>
+        <v>0.84983</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8.4983</v>
+      </c>
+      <c r="E3" t="n">
+        <v>84.983</v>
+      </c>
+      <c r="F3" t="n">
+        <v>849.83</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>INR</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>100</v>
-      </c>
       <c r="C4" t="n">
-        <v>9282</v>
+        <v>93.51000000000001</v>
+      </c>
+      <c r="D4" t="n">
+        <v>935.1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>9351</v>
+      </c>
+      <c r="F4" t="n">
+        <v>93510</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>INR</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1000</v>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AUD</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>92820</v>
+        <v>1.3957</v>
+      </c>
+      <c r="D5" t="n">
+        <v>13.957</v>
+      </c>
+      <c r="E5" t="n">
+        <v>139.57</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1395.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CAD</t>
+        </is>
       </c>
       <c r="C6" t="n">
-        <v>1.3934</v>
+        <v>1.3657</v>
+      </c>
+      <c r="D6" t="n">
+        <v>13.657</v>
+      </c>
+      <c r="E6" t="n">
+        <v>136.57</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1365.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>10</v>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>JPY</t>
+        </is>
       </c>
       <c r="C7" t="n">
-        <v>13.934</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>100</v>
-      </c>
-      <c r="C8" t="n">
-        <v>139.34</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>AUD</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C9" t="n">
-        <v>1393.4</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" t="n">
-        <v>1.3672</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>10</v>
-      </c>
-      <c r="C11" t="n">
-        <v>13.672</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>100</v>
-      </c>
-      <c r="C12" t="n">
-        <v>136.72</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>CAD</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C13" t="n">
-        <v>1367.2</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0.84767</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>10</v>
-      </c>
-      <c r="C15" t="n">
-        <v>8.476700000000001</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>100</v>
-      </c>
-      <c r="C16" t="n">
-        <v>84.76700000000001</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C17" t="n">
-        <v>847.6700000000001</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.7389</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>10</v>
-      </c>
-      <c r="C19" t="n">
-        <v>7.389</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>100</v>
-      </c>
-      <c r="C20" t="n">
-        <v>73.89</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C21" t="n">
-        <v>738.9</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>JPY</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="n">
-        <v>159.13</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>JPY</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>10</v>
-      </c>
-      <c r="C23" t="n">
-        <v>1591.3</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>JPY</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>100</v>
-      </c>
-      <c r="C24" t="n">
-        <v>15913</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>JPY</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C25" t="n">
-        <v>159130</v>
+        <v>159.04</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1590.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>15904</v>
+      </c>
+      <c r="F7" t="n">
+        <v>159040</v>
       </c>
     </row>
   </sheetData>

</xml_diff>